<commit_message>
Add synthetic study response demo
</commit_message>
<xml_diff>
--- a/study/analysis/mathontospeak_study_analysis_template.xlsx
+++ b/study/analysis/mathontospeak_study_analysis_template.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R65c5d909e716428b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="2" r:id="R11b92adc27144ee7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counterbalance" sheetId="3" r:id="R5369240f72084b3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comprehension Scores" sheetId="4" r:id="R53f84dca5a5e490d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NASA TLX" sheetId="5" r:id="Re6d3cca6a4364e35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCQ Items" sheetId="6" r:id="R639f6200da1741aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview Coding" sheetId="7" r:id="Re2a8af84fb1a487c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R337ad519ee7a4e18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="2" r:id="Rded8e00c62d54d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counterbalance" sheetId="3" r:id="R092ce785379d4677"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comprehension Scores" sheetId="4" r:id="Rc78910ce283f4eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NASA TLX" sheetId="5" r:id="Read54589d39042d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCQ Items" sheetId="6" r:id="R692cb2ed1c614b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview Coding" sheetId="7" r:id="R5c7b4c19f76249e3"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>